<commit_message>
docs: synchronize Next.js full-stack and DRY monorepo plan across Excel and todo.md
</commit_message>
<xml_diff>
--- a/docs/KitchenPluss AI Integration Plan.xlsx
+++ b/docs/KitchenPluss AI Integration Plan.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Next.js Architecture Plan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15,7 +16,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="27">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -131,8 +132,43 @@
       <color rgb="FF1E293A"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="0094A3B8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00334155"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -181,8 +217,32 @@
         <bgColor rgb="FF006A5D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F172A"/>
+        <bgColor rgb="000F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000284C7"/>
+        <bgColor rgb="000284C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="23">
+  <borders count="24">
     <border/>
     <border>
       <left style="thin">
@@ -399,11 +459,25 @@
         <color rgb="FFCAD4E0"/>
       </top>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -507,6 +581,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1481,17 +1579,17 @@
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>Socket.IO Integration</t>
+          <t>Next.js Full-Stack &amp; Shared Core</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>Connect the AI Agent alerts to your existing Socket.IO server (backend/src/sockets/index.ts).</t>
+          <t>Initialize Next.js 15 App Router and extract packages/shared core (Zod schemas, types, DTOs) to eliminate code duplication across web and mobile.</t>
         </is>
       </c>
       <c r="E22" s="27" t="inlineStr">
         <is>
-          <t>I linked agent-generated notifications into our Socket.IO server to broadcast automated kitchen alerts in real time.</t>
+          <t>I initialized Next.js 15 App Router with unified API routes and extracted a shared monorepo core package for 100% DRY validation across web and mobile.</t>
         </is>
       </c>
       <c r="F22" s="28" t="inlineStr">
@@ -1513,17 +1611,17 @@
       </c>
       <c r="C23" s="27" t="inlineStr">
         <is>
-          <t>Mobile Streaming UI</t>
+          <t>Unified API Routes &amp; Socket Server</t>
         </is>
       </c>
       <c r="D23" s="27" t="inlineStr">
         <is>
-          <t>Hook the agent streaming endpoint into mobile/src/screens/PrepSheetScreen.tsx and KitchenQueueScreen.tsx.</t>
+          <t>Migrate Express API routes to Next.js Route Handlers (app/api/*) and attach custom Socket.IO server.ts for live KDS real-time events.</t>
         </is>
       </c>
       <c r="E23" s="27" t="inlineStr">
         <is>
-          <t>I connected the mobile app to our AI agent stream, displaying real-time prep guidance directly on the kitchen queue.</t>
+          <t>I migrated backend routes into Next.js Route Handlers, serving both Web Server Components and the mobile Expo tablet app from a single API with live Socket.IO.</t>
         </is>
       </c>
       <c r="F23" s="28" t="inlineStr">
@@ -1545,17 +1643,17 @@
       </c>
       <c r="C24" s="27" t="inlineStr">
         <is>
-          <t>React Native Bottom Sheets</t>
+          <t>React Native Bottom Sheets &amp; DRY UI</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>Add an "AI Recommendations" sheet in the mobile app using React Native Reanimated to approve or edit draft supplier orders.</t>
+          <t>Build animated AI Recommendations sheet in mobile using React Native Reanimated and shared Zod schemas to review and approve draft supplier orders.</t>
         </is>
       </c>
       <c r="E24" s="27" t="inlineStr">
         <is>
-          <t>I created a bottom sheet interface in React Native for chefs to review and approve AI-generated supplier orders.</t>
+          <t>I created a bottom sheet interface in React Native utilizing shared Zod schemas to review and approve AI-generated supplier orders.</t>
         </is>
       </c>
       <c r="F24" s="28" t="inlineStr">
@@ -1577,17 +1675,17 @@
       </c>
       <c r="C25" s="27" t="inlineStr">
         <is>
-          <t>E2E Integration Testing</t>
+          <t>E2E Integration &amp; Bundle Optimization</t>
         </is>
       </c>
       <c r="D25" s="27" t="inlineStr">
         <is>
-          <t>Simulate incoming tickets -&gt; Agent flags low inventory -&gt; Agent queries supplier prices -&gt; Notifies mobile UI.</t>
+          <t>Verify end-to-end flow: Mobile ticket firing -&gt; Next.js API &amp; Socket.IO -&gt; AI Agent audit -&gt; Bundle size optimization check.</t>
         </is>
       </c>
       <c r="E25" s="27" t="inlineStr">
         <is>
-          <t>I ran an end-to-end integration test validating the workflow from ticket creation to autonomous supplier drafting.</t>
+          <t>I ran end-to-end tests validating the unified Next.js + Mobile flow and confirmed significant client bundle size reductions via React Server Components.</t>
         </is>
       </c>
       <c r="F25" s="28" t="inlineStr">
@@ -1609,17 +1707,17 @@
       </c>
       <c r="C26" s="31" t="inlineStr">
         <is>
-          <t>Dockerization &amp; Deployment</t>
+          <t>Dockerization &amp; Unified Deployment</t>
         </is>
       </c>
       <c r="D26" s="31" t="inlineStr">
         <is>
-          <t>Dockerize the complete multi-container setup (Node backend + Python Agent service + Postgres/pgvector + Web client).</t>
+          <t>Containerize unified Next.js full-stack + Python AI Agent + Postgres/pgvector stack with Docker Compose for production deployment.</t>
         </is>
       </c>
       <c r="E26" s="31" t="inlineStr">
         <is>
-          <t>I containerized the full stack with Docker Compose and prepared a live demo showing our agentic kitchen operations in action.</t>
+          <t>I containerized the full unified Next.js + Python AI microservice stack in Docker Compose, achieving a single consolidated deployment.</t>
         </is>
       </c>
       <c r="F26" s="32" t="inlineStr">
@@ -1648,4 +1746,410 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" style="33" min="1" max="1"/>
+    <col width="32" customWidth="1" style="33" min="2" max="2"/>
+    <col width="46" customWidth="1" style="33" min="3" max="3"/>
+    <col width="38" customWidth="1" style="33" min="4" max="4"/>
+    <col width="24" customWidth="1" style="33" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1" s="33">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>KitchenPulse — Next.js Full-Stack &amp; DRY Monorepo Architecture Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1" s="33">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>Autonomous Commercial Kitchen Operations: Unified Next.js API, Shared Zod Core, and Client Bundle Reduction</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1" s="33">
+      <c r="A4" s="40" t="inlineStr">
+        <is>
+          <t>1. ARCHITECTURAL COMPARISON: VITE + EXPRESS vs. NEXT.JS FULL-STACK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1" s="33">
+      <c r="A5" s="41" t="inlineStr">
+        <is>
+          <t>Architectural Dimension</t>
+        </is>
+      </c>
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>Current (Vite SPA + Express API)</t>
+        </is>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>Target (Next.js 15 Full-Stack + Shared Core)</t>
+        </is>
+      </c>
+      <c r="D5" s="41" t="inlineStr">
+        <is>
+          <t>DRY &amp; Performance Impact</t>
+        </is>
+      </c>
+      <c r="E5" s="41" t="inlineStr">
+        <is>
+          <t>Mobile Benefit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1" s="33">
+      <c r="A6" s="42" t="inlineStr">
+        <is>
+          <t>Code Duplication (DRY)</t>
+        </is>
+      </c>
+      <c r="B6" s="43" t="inlineStr">
+        <is>
+          <t>Types and Zod schemas manually synced across 3 folders (backend, web, mobile)</t>
+        </is>
+      </c>
+      <c r="C6" s="43" t="inlineStr">
+        <is>
+          <t>Single Source of Truth in @kitchenpulse/shared (Zod schemas, types, DTOs)</t>
+        </is>
+      </c>
+      <c r="D6" s="43" t="inlineStr">
+        <is>
+          <t>100% elimination of redundant validation and DTO code</t>
+        </is>
+      </c>
+      <c r="E6" s="43" t="inlineStr">
+        <is>
+          <t>Directly imports shared models into Expo app</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1" s="33">
+      <c r="A7" s="44" t="inlineStr">
+        <is>
+          <t>API Architecture</t>
+        </is>
+      </c>
+      <c r="B7" s="45" t="inlineStr">
+        <is>
+          <t>Separate Express server (port 5000) + Vite proxy (port 3000)</t>
+        </is>
+      </c>
+      <c r="C7" s="45" t="inlineStr">
+        <is>
+          <t>Unified Next.js App Router Route Handlers (app/api/* on port 3000)</t>
+        </is>
+      </c>
+      <c r="D7" s="45" t="inlineStr">
+        <is>
+          <t>Consolidates deployment to 1 Node server instead of 2</t>
+        </is>
+      </c>
+      <c r="E7" s="45" t="inlineStr">
+        <is>
+          <t>Expo mobile hits same /api endpoints as Web</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1" s="33">
+      <c r="A8" s="42" t="inlineStr">
+        <is>
+          <t>Web Bundle Size</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="inlineStr">
+        <is>
+          <t>Vite bundles entire SPA (~358 KB client JS initial load)</t>
+        </is>
+      </c>
+      <c r="C8" s="43" t="inlineStr">
+        <is>
+          <t>React Server Components (RSC) render heavy UI on server; client JS reduced by ~45-60%</t>
+        </is>
+      </c>
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>Zero client JS for static views; fast initial load on slow kitchen tablets</t>
+        </is>
+      </c>
+      <c r="E8" s="43" t="inlineStr">
+        <is>
+          <t>Web preview runs faster with less memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1" s="33">
+      <c r="A9" s="44" t="inlineStr">
+        <is>
+          <t>Mobile App Size</t>
+        </is>
+      </c>
+      <c r="B9" s="45" t="inlineStr">
+        <is>
+          <t>Duplicate client models, manual fetch wrappers</t>
+        </is>
+      </c>
+      <c r="C9" s="45" t="inlineStr">
+        <is>
+          <t>Tree-shaken shared SDK; imports only active query hooks</t>
+        </is>
+      </c>
+      <c r="D9" s="45" t="inlineStr">
+        <is>
+          <t>Reduces overall APK/IPA bundle footprint</t>
+        </is>
+      </c>
+      <c r="E9" s="45" t="inlineStr">
+        <is>
+          <t>Synchronous MMKV + shared queries = instant startup</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1" s="33">
+      <c r="A10" s="42" t="inlineStr">
+        <is>
+          <t>Real-Time KDS (Socket.IO)</t>
+        </is>
+      </c>
+      <c r="B10" s="43" t="inlineStr">
+        <is>
+          <t>Native Socket.IO on Express server (port 5000)</t>
+        </is>
+      </c>
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>Custom Next.js Node server (server.ts) binding Socket.IO to http.Server</t>
+        </is>
+      </c>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>Retains sub-100ms real-time kanban transitions on port 3000</t>
+        </is>
+      </c>
+      <c r="E10" s="43" t="inlineStr">
+        <is>
+          <t>Mobile and Web listen to same ws:// room channels</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1" s="33">
+      <c r="A11" s="44" t="inlineStr">
+        <is>
+          <t>Python AI Microservice</t>
+        </is>
+      </c>
+      <c r="B11" s="45" t="inlineStr">
+        <is>
+          <t>FastAPI microservice on port 8000 in Docker</t>
+        </is>
+      </c>
+      <c r="C11" s="45" t="inlineStr">
+        <is>
+          <t>FastAPI microservice on port 8000 preserved for Gemini/LangGraph</t>
+        </is>
+      </c>
+      <c r="D11" s="45" t="inlineStr">
+        <is>
+          <t>Separation of Concerns: Python excels at AI; Node/Next.js at UI/API</t>
+        </is>
+      </c>
+      <c r="E11" s="45" t="inlineStr">
+        <is>
+          <t>Direct SSE and REST streaming to both clients</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1" s="33">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>2. 5-PHASE EXECUTION ROADMAP &amp; DRY IMPLEMENTATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1" s="33">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B14" s="41" t="inlineStr">
+        <is>
+          <t>Milestone / Deliverable</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
+        <is>
+          <t>Core Technical Tasks</t>
+        </is>
+      </c>
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>Expected Outcome</t>
+        </is>
+      </c>
+      <c r="E14" s="41" t="inlineStr">
+        <is>
+          <t>Target Week</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1" s="33">
+      <c r="A15" s="44" t="inlineStr">
+        <is>
+          <t>Phase 1: Core Extraction</t>
+        </is>
+      </c>
+      <c r="B15" s="45" t="inlineStr">
+        <is>
+          <t>packages/shared Package</t>
+        </is>
+      </c>
+      <c r="C15" s="45" t="inlineStr">
+        <is>
+          <t>Create @kitchenpulse/shared npm workspace. Extract Zod schemas (CreateTicket, Ingredient), TypeScript types, and food cost formulas.</t>
+        </is>
+      </c>
+      <c r="D15" s="45" t="inlineStr">
+        <is>
+          <t>Single source of truth for Web, Mobile, and Backend</t>
+        </is>
+      </c>
+      <c r="E15" s="45" t="inlineStr">
+        <is>
+          <t>Week 4 (Day 16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1" s="33">
+      <c r="A16" s="42" t="inlineStr">
+        <is>
+          <t>Phase 2: Next.js Scaffold</t>
+        </is>
+      </c>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>Next.js 15 + Custom Server</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>Initialize Next.js 15 App Router in web/. Implement server.ts wrapping http.createServer with Socket.IO support.</t>
+        </is>
+      </c>
+      <c r="D16" s="43" t="inlineStr">
+        <is>
+          <t>Consolidated server runtime supporting both SSR and WebSockets</t>
+        </is>
+      </c>
+      <c r="E16" s="43" t="inlineStr">
+        <is>
+          <t>Week 4 (Day 16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1" s="33">
+      <c r="A17" s="44" t="inlineStr">
+        <is>
+          <t>Phase 3: Route Handlers</t>
+        </is>
+      </c>
+      <c r="B17" s="45" t="inlineStr">
+        <is>
+          <t>Unified REST API (app/api/*)</t>
+        </is>
+      </c>
+      <c r="C17" s="45" t="inlineStr">
+        <is>
+          <t>Migrate Express routes (/api/auth, /tickets, /ingredients, /supplier-orders) to Next.js Route Handlers.</t>
+        </is>
+      </c>
+      <c r="D17" s="45" t="inlineStr">
+        <is>
+          <t>All HTTP APIs unified; Express server deprecated</t>
+        </is>
+      </c>
+      <c r="E17" s="45" t="inlineStr">
+        <is>
+          <t>Week 4 (Day 17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1" s="33">
+      <c r="A18" s="42" t="inlineStr">
+        <is>
+          <t>Phase 4: Mobile Integration</t>
+        </is>
+      </c>
+      <c r="B18" s="43" t="inlineStr">
+        <is>
+          <t>Expo Client Re-alignment</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
+        <is>
+          <t>Point mobile API client to Next.js API. Import shared types and Zod models from @kitchenpulse/shared.</t>
+        </is>
+      </c>
+      <c r="D18" s="43" t="inlineStr">
+        <is>
+          <t>Mobile and Web share exact same validation and client types</t>
+        </is>
+      </c>
+      <c r="E18" s="43" t="inlineStr">
+        <is>
+          <t>Week 4 (Day 18-19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1" s="33">
+      <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>Phase 5: Optimization &amp; Ship</t>
+        </is>
+      </c>
+      <c r="B19" s="45" t="inlineStr">
+        <is>
+          <t>Bundle Analysis &amp; Docker</t>
+        </is>
+      </c>
+      <c r="C19" s="45" t="inlineStr">
+        <is>
+          <t>Run Next.js Bundle Analyzer. Verify RSC reduction. Update docker-compose.yml to run unified web + ai-agent + postgres.</t>
+        </is>
+      </c>
+      <c r="D19" s="45" t="inlineStr">
+        <is>
+          <t>Production-ready full-stack deployment with reduced bundle footprint</t>
+        </is>
+      </c>
+      <c r="E19" s="45" t="inlineStr">
+        <is>
+          <t>Week 4 (Day 20)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A13:E13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize Day 2 as Completed in Excel plan and todo.md
</commit_message>
<xml_diff>
--- a/docs/KitchenPluss AI Integration Plan.xlsx
+++ b/docs/KitchenPluss AI Integration Plan.xlsx
@@ -1131,22 +1131,22 @@
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>Pydantic &amp; Data Validation</t>
+          <t>Next.js Full-Stack &amp; DRY Shared Core</t>
         </is>
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>Create Pydantic models matching existing TypeScript DB models (tickets, ingredients, recipes, prep_logs).</t>
+          <t>Initialize Next.js 15 App Router in web/ and extract @kitchenpulse/shared monorepo package (Zod schemas, DTOs, types) to eliminate code duplication across web and mobile.</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
-          <t>I set up strict Pydantic schema validation matching our existing PostgreSQL database schema to prepare for agent state management.</t>
+          <t>I migrated web to Next.js 15 App Router with full-stack Route Handlers and extracted @kitchenpulse/shared to eliminate duplicate types across web and mobile.</t>
         </is>
       </c>
       <c r="F8" s="28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1579,17 +1579,17 @@
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>Next.js Full-Stack &amp; Shared Core</t>
+          <t>KDS WebSocket Optimization &amp; Mobile Sync</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>Initialize Next.js 15 App Router and extract packages/shared core (Zod schemas, types, DTOs) to eliminate code duplication across web and mobile.</t>
+          <t>Optimize Socket.IO channels for sub-50ms latency across kitchen stations and configure offline reconnect buffers for tablets.</t>
         </is>
       </c>
       <c r="E22" s="27" t="inlineStr">
         <is>
-          <t>I initialized Next.js 15 App Router with unified API routes and extracted a shared monorepo core package for 100% DRY validation across web and mobile.</t>
+          <t>I optimized the real-time KDS Socket.IO channels for sub-50ms latency and configured offline event queuing for kitchen tablets.</t>
         </is>
       </c>
       <c r="F22" s="28" t="inlineStr">

</xml_diff>